<commit_message>
feat: add control tower workflow follow through
</commit_message>
<xml_diff>
--- a/bof-web/public/data/main-source-v4_operational_elite_enhanced.xlsx
+++ b/bof-web/public/data/main-source-v4_operational_elite_enhanced.xlsx
@@ -33280,7 +33280,7 @@
         <v>HOLD-003</v>
       </c>
       <c r="H4" t="str">
-        <v>Missing lumper receipt</v>
+        <v>QR lumper authorization closeout pending</v>
       </c>
       <c r="I4" t="str">
         <v>Medium</v>
@@ -33289,13 +33289,13 @@
         <v>Open</v>
       </c>
       <c r="K4" t="str">
-        <v>Accessorial reimbursement cannot be closed</v>
+        <v>Accessorial closeout waits on dock-side QR authorization, empty-trailer proof, and Zelle payment confirmation</v>
       </c>
       <c r="L4" t="str">
         <v>Eligible</v>
       </c>
       <c r="M4" t="str">
-        <v>$180 hold</v>
+        <v>$180 closeout hold</v>
       </c>
       <c r="N4" t="str">
         <v>None</v>
@@ -33310,7 +33310,7 @@
         <v>Settlement Desk</v>
       </c>
       <c r="R4" t="str">
-        <v>Upload lumper receipt or mark not required with dispatcher approval</v>
+        <v>Match QR dock authorization, empty-trailer proof, and Zelle payment confirmation to release accessorial closeout</v>
       </c>
       <c r="S4" t="str">
         <v>Open</v>
@@ -33319,7 +33319,7 @@
         <v/>
       </c>
       <c r="U4" t="str">
-        <v>Resolve missing receipt</v>
+        <v>Review QR lumper closeout</v>
       </c>
     </row>
   </sheetData>
@@ -33904,16 +33904,16 @@
         <v>L-507</v>
       </c>
       <c r="F4" t="str">
-        <v>Receipt Hold</v>
+        <v>QR Lumper Closeout</v>
       </c>
       <c r="G4" t="str">
-        <v>Lumper receipt missing for reimbursement</v>
+        <v>QR lumper authorization and Zelle payment closeout pending</v>
       </c>
       <c r="H4" t="str">
-        <v>Settlement/Documents</v>
+        <v>Settlements</v>
       </c>
       <c r="I4" t="str">
-        <v>DOC-507-LUMPER</v>
+        <v>LUMPER-QR-507</v>
       </c>
       <c r="J4">
         <v>180</v>
@@ -33934,7 +33934,7 @@
         <v/>
       </c>
       <c r="P4" t="str">
-        <v>Upload lumper receipt</v>
+        <v>Review QR lumper closeout</v>
       </c>
     </row>
   </sheetData>
@@ -35871,7 +35871,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:ED13"/>
+  <dimension ref="A1:EG13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -36276,6 +36276,15 @@
       <c r="ED1" t="str">
         <v>Settlement Release Date</v>
       </c>
+      <c r="EE1" t="str">
+        <v>Settlement Hold</v>
+      </c>
+      <c r="EF1" t="str">
+        <v>Document Status</v>
+      </c>
+      <c r="EG1" t="str">
+        <v>Exception Reason</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -39021,7 +39030,7 @@
         <v>YES</v>
       </c>
       <c r="DC8" t="str">
-        <v>Missing lumper receipt for reimbursement</v>
+        <v>QR lumper authorization and Zelle payment closeout pending</v>
       </c>
       <c r="DD8" t="str">
         <v>NEEDS_REVIEW</v>
@@ -39103,6 +39112,15 @@
       </c>
       <c r="ED8" t="str">
         <v/>
+      </c>
+      <c r="EE8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="EF8" t="str">
+        <v>NEEDS_REVIEW</v>
+      </c>
+      <c r="EG8" t="str">
+        <v>QR lumper authorization/payment closeout pending</v>
       </c>
     </row>
     <row r="9">
@@ -41127,7 +41145,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:ED13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:EG13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>